<commit_message>
Initial exploration - understanding codebase structure
Agent-Logs-Url: https://github.com/Braumeister-Stefan/lina_database_builder/sessions/3cf4e3a2-ae59-4465-852b-c958b0af539a

Co-authored-by: Braumeister-Stefan <80990521+Braumeister-Stefan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/lina_report.xlsx
+++ b/data/lina_report.xlsx
@@ -392,7 +392,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="6048375"/>
+    <ext cx="10477500" cy="5686425"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -15438,11 +15438,11 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tablet Find-Sites – Aegean Region</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="476.25" customHeight="1"/>
+          <t>Tablet Find-Sites – Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="447.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Replace Crete polygon with geographic map, add quality confidence scoring and inclusion strategy
Agent-Logs-Url: https://github.com/Braumeister-Stefan/lina_database_builder/sessions/3cf4e3a2-ae59-4465-852b-c958b0af539a

Co-authored-by: Braumeister-Stefan <80990521+Braumeister-Stefan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/lina_report.xlsx
+++ b/data/lina_report.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Timeline" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Signs per Tablet" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Coverage" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Quality" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -233,6 +234,36 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="12496800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -392,7 +423,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="5686425"/>
+    <ext cx="10477500" cy="8553450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -15438,11 +15469,11 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tablet Find-Sites – Crete</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="447.75" customHeight="1"/>
+          <t>Tablet Find-Sites – Crete &amp; Aegean</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="673.5" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -15512,6 +15543,29 @@
       </c>
     </row>
     <row r="2" ht="795.75" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source Quality Confidence Scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="984" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Initial exploration - no changes yet
Agent-Logs-Url: https://github.com/Braumeister-Stefan/lina_database_builder/sessions/1dc9af4b-d38e-4d35-9bc4-91b922cb4a45

Co-authored-by: Braumeister-Stefan <80990521+Braumeister-Stefan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/lina_report.xlsx
+++ b/data/lina_report.xlsx
@@ -392,7 +392,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="6048375"/>
+    <ext cx="10477500" cy="5686425"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -15438,11 +15438,11 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tablet Find-Sites – Aegean Region</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="476.25" customHeight="1"/>
+          <t>Tablet Find-Sites – Crete</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="447.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>